<commit_message>
spatial density analysis of conflicts,
</commit_message>
<xml_diff>
--- a/data_base_overview.xlsx
+++ b/data_base_overview.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Documents\DCRM\DCRM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08101CCB-BB44-4757-9085-04F1C9A91328}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE3C52CF-09F1-4711-BF4C-4912CB13D9A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2205" yWindow="2205" windowWidth="16875" windowHeight="10523" xr2:uid="{04E4B17E-71F9-4E6D-BF73-45AE3ECF8B19}"/>
+    <workbookView xWindow="2940" yWindow="2940" windowWidth="16875" windowHeight="10522" xr2:uid="{04E4B17E-71F9-4E6D-BF73-45AE3ECF8B19}"/>
   </bookViews>
   <sheets>
     <sheet name="input" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="44">
   <si>
     <t>Topic</t>
   </si>
@@ -161,6 +161,15 @@
   </si>
   <si>
     <t>see doc in folder structure</t>
+  </si>
+  <si>
+    <t>EJAtlas_dataset_V1_2024-01.xlsx</t>
+  </si>
+  <si>
+    <t>EJAtlas</t>
+  </si>
+  <si>
+    <t>Scheidel et al., 2023</t>
   </si>
 </sst>
 </file>
@@ -526,13 +535,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CB9D47A-77E7-41F3-B04A-F56D03723ECC}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="30.06640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28.53125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="24.19921875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.46484375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="23.86328125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="30.33203125" bestFit="1" customWidth="1"/>
   </cols>
@@ -684,6 +693,20 @@
         <v>39</v>
       </c>
       <c r="D9" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C10" t="s">
+        <v>43</v>
+      </c>
+      <c r="D10" t="s">
         <v>40</v>
       </c>
     </row>

</xml_diff>